<commit_message>
Remove MoreTasks and C11 Aura from outreach tracker
Both rejected the application; dropping them from the active list.
Tracker rebuilt from source: 13 rows to 11.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TsefmjrgrWVU5PNpRHnLLk
</commit_message>
<xml_diff>
--- a/outreach/Outreach_Tracker.xlsx
+++ b/outreach/Outreach_Tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outreach" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do Not Contact" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Outreach" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Do Not Contact" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="How to use" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X14"/>
+  <dimension ref="A1:X12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -672,42 +672,42 @@
       <c r="A2" s="2" t="inlineStr"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>MoreTasks</t>
+          <t>The Bijou Box</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>moretasks.com</t>
+          <t>thebijoubox.in</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Business Services / Ops</t>
+          <t>D2C / Jewellery</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Growth</t>
+          <t>Early</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Delhi NCR</t>
+          <t>Mumbai</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Gauri Chaturvedi</t>
+          <t>Hiring Team</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Talent Acquisition</t>
+          <t>Founder / Hiring</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>gauri.chaturvedi@moretasks.com</t>
+          <t>info@thebijoubox.in</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -722,7 +722,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Operations Manager</t>
+          <t>E-commerce Operations</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr"/>
@@ -754,7 +754,7 @@
       </c>
       <c r="X2" s="3" t="inlineStr">
         <is>
-          <t>P1. Chased twice for Business Ops Associate, left callback 9205888799. Also cc: priyanshi.agarwal@moretasks.com, somya.devvanshi@moretasks.com</t>
+          <t>P1. Said "CV aligns well with our requirements", booked a call, then went quiet. Requires Mumbai relocation.</t>
         </is>
       </c>
     </row>
@@ -762,13 +762,17 @@
       <c r="A3" s="2" t="inlineStr"/>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>C11 Aura</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr"/>
+          <t>Gudz</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>gudz.in</t>
+        </is>
+      </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Consumer / Retail</t>
+          <t>D2C / Consumer</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -778,27 +782,27 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Kharar, Mohali</t>
+          <t>Gurugram (Sector 49)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Navjot Kaur</t>
+          <t>Aryaman</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Recruiter</t>
+          <t>Founder</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>navjotkaurwork123@gmail.com</t>
+          <t>aryaman@gudz.in</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Gmail - inbound Jul 2026</t>
+          <t>Gmail - inbound May 2026</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -808,7 +812,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Operations Lead</t>
+          <t>Operations Manager</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -840,7 +844,7 @@
       </c>
       <c r="X3" s="3" t="inlineStr">
         <is>
-          <t>P1. Shortlisted for Ops Lead Round 2; interview missed (family emergency), they rescheduled 28 Jul. Closest role match to target.</t>
+          <t>P1. Replied same day, offered walk-in. Earlier role was fresher-level; re-approach at manager level. cc: darshan@gudz.in</t>
         </is>
       </c>
     </row>
@@ -848,47 +852,47 @@
       <c r="A4" s="2" t="inlineStr"/>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>The Bijou Box</t>
+          <t>Meesho</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>thebijoubox.in</t>
+          <t>meesho.com</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>D2C / Jewellery</t>
+          <t>E-commerce Marketplace</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Early</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Mumbai</t>
+          <t>Panipat / NCR</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Hiring Team</t>
+          <t>Sharukh Khan</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Founder / Hiring</t>
+          <t>Recruiter</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>info@thebijoubox.in</t>
+          <t>sharukh.khan1@meesho.com</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Gmail - inbound May 2026</t>
+          <t>Gmail - Apr/May 2026</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -898,7 +902,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>E-commerce Operations</t>
+          <t>Area Manager / Ops</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr"/>
@@ -930,7 +934,7 @@
       </c>
       <c r="X4" s="3" t="inlineStr">
         <is>
-          <t>P1. Said "CV aligns well with our requirements", booked a call, then went quiet. Requires Mumbai relocation.</t>
+          <t>P1. Area Manager process was live via mynexthire; asked for update, no reply. Worth reopening.</t>
         </is>
       </c>
     </row>
@@ -938,17 +942,17 @@
       <c r="A5" s="2" t="inlineStr"/>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Gudz</t>
+          <t>Elda</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>gudz.in</t>
+          <t>getelda.com</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>D2C / Consumer</t>
+          <t>Consumer Internet</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -956,14 +960,10 @@
           <t>Early</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Gurugram (Sector 49)</t>
-        </is>
-      </c>
+      <c r="F5" s="2" t="inlineStr"/>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Aryaman</t>
+          <t>Jayant</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -973,12 +973,12 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>aryaman@gudz.in</t>
+          <t>jayant@getelda.com</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Gmail - inbound May 2026</t>
+          <t>Gmail - inbound Jul 2026</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Operations Manager</t>
+          <t>Business Operations</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr"/>
@@ -1020,183 +1020,179 @@
       </c>
       <c r="X5" s="3" t="inlineStr">
         <is>
-          <t>P1. Replied same day, offered walk-in. Earlier role was fresher-level; re-approach at manager level. cc: darshan@gudz.in</t>
+          <t>P1. Sent Founder's Office JD in Jul 2026. Was intern-level; ask about full-time ops.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Meesho</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>meesho.com</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>E-commerce Marketplace</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Panipat / NCR</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Sharukh Khan</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Recruiter</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>sharukh.khan1@meesho.com</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>Gmail - Apr/May 2026</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>Warm</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>Area Manager / Ops</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr"/>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O6" s="2" t="inlineStr"/>
-      <c r="P6" s="2" t="inlineStr"/>
-      <c r="Q6" s="2" t="inlineStr"/>
-      <c r="R6" s="2" t="inlineStr"/>
-      <c r="S6" s="2" t="inlineStr"/>
-      <c r="T6" s="2" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr"/>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Cameron SF</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>cameronsf.com</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>D2C / Consumer</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Early</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr"/>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Justin</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>justin@cameronsf.com</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>Gmail - outbound May 2026</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>Operations Manager</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="inlineStr"/>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O6" s="4" t="inlineStr"/>
+      <c r="P6" s="4" t="inlineStr"/>
+      <c r="Q6" s="4" t="inlineStr"/>
+      <c r="R6" s="4" t="inlineStr"/>
+      <c r="S6" s="4" t="inlineStr"/>
+      <c r="T6" s="4" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="U6" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="V6" s="2" t="inlineStr"/>
-      <c r="W6" s="2" t="inlineStr">
+      <c r="U6" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V6" s="4" t="inlineStr"/>
+      <c r="W6" s="4" t="inlineStr">
         <is>
           <t>Ready to Send</t>
         </is>
       </c>
-      <c r="X6" s="3" t="inlineStr">
-        <is>
-          <t>P1. Area Manager process was live via mynexthire; asked for update, no reply. Worth reopening.</t>
+      <c r="X6" s="5" t="inlineStr">
+        <is>
+          <t>P3. Applied for Operations Manager May 2026, no reply. Verify company still active before re-sending.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr"/>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Elda</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>getelda.com</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Consumer Internet</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr"/>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Zoomuv</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>zoomuv.com</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Logistics / Mobility</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>Early</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Jayant</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr"/>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Dheeraj Gupta</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>Founder</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>jayant@getelda.com</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>Gmail - inbound Jul 2026</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>Warm</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>Business Operations</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr"/>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O7" s="2" t="inlineStr"/>
-      <c r="P7" s="2" t="inlineStr"/>
-      <c r="Q7" s="2" t="inlineStr"/>
-      <c r="R7" s="2" t="inlineStr"/>
-      <c r="S7" s="2" t="inlineStr"/>
-      <c r="T7" s="2" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>dheeraj@zoomuv.com</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>Gmail - outbound May 2026</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>Operations Executive</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="inlineStr"/>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O7" s="4" t="inlineStr"/>
+      <c r="P7" s="4" t="inlineStr"/>
+      <c r="Q7" s="4" t="inlineStr"/>
+      <c r="R7" s="4" t="inlineStr"/>
+      <c r="S7" s="4" t="inlineStr"/>
+      <c r="T7" s="4" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="U7" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="V7" s="2" t="inlineStr"/>
-      <c r="W7" s="2" t="inlineStr">
+      <c r="U7" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V7" s="4" t="inlineStr"/>
+      <c r="W7" s="4" t="inlineStr">
         <is>
           <t>Ready to Send</t>
         </is>
       </c>
-      <c r="X7" s="3" t="inlineStr">
-        <is>
-          <t>P1. Sent Founder's Office JD in Jul 2026. Was intern-level; ask about full-time ops.</t>
+      <c r="X7" s="5" t="inlineStr">
+        <is>
+          <t>P3. Applied May 2026, no reply.</t>
         </is>
       </c>
     </row>
@@ -1204,38 +1200,42 @@
       <c r="A8" s="4" t="inlineStr"/>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Cameron SF</t>
+          <t>Ugaoo</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>cameronsf.com</t>
+          <t>ugaoo.com</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>D2C / Consumer</t>
+          <t>D2C / Plants</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Early</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr"/>
+          <t>Growth</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Pune</t>
+        </is>
+      </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Justin</t>
+          <t>Shubham S</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Founder</t>
+          <t>Hiring Manager</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>justin@cameronsf.com</t>
+          <t>shubham.s@ugaoo.com</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -1282,7 +1282,7 @@
       </c>
       <c r="X8" s="5" t="inlineStr">
         <is>
-          <t>P3. Applied for Operations Manager May 2026, no reply. Verify company still active before re-sending.</t>
+          <t>P2. Applied for Manager - Process Excellence May 2026. Established D2C, strong fit.</t>
         </is>
       </c>
     </row>
@@ -1290,17 +1290,17 @@
       <c r="A9" s="4" t="inlineStr"/>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Zoomuv</t>
+          <t>Samplify</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>zoomuv.com</t>
+          <t>gosamplify.com</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Logistics / Mobility</t>
+          <t>D2C / Sampling</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -1311,17 +1311,17 @@
       <c r="F9" s="4" t="inlineStr"/>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Dheeraj Gupta</t>
+          <t>Hemlata</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Founder</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>dheeraj@zoomuv.com</t>
+          <t>hemlata@gosamplify.com</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1336,7 +1336,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>Operations Executive</t>
+          <t>Team Lead - Operations</t>
         </is>
       </c>
       <c r="M9" s="4" t="inlineStr"/>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="X9" s="5" t="inlineStr">
         <is>
-          <t>P3. Applied May 2026, no reply.</t>
+          <t>P2. Applied May 2026, no reply.</t>
         </is>
       </c>
     </row>
@@ -1376,42 +1376,38 @@
       <c r="A10" s="4" t="inlineStr"/>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Ugaoo</t>
+          <t>goPortals</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>ugaoo.com</t>
+          <t>goportals.co</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>D2C / Plants</t>
+          <t>E-commerce</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Growth</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>Pune</t>
-        </is>
-      </c>
+          <t>Early</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr"/>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Shubham S</t>
+          <t>Sahil Gupta</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Hiring Manager</t>
+          <t>Founder</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>shubham.s@ugaoo.com</t>
+          <t>sahilgupta@goportals.co</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1426,7 +1422,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>Operations Manager</t>
+          <t>E-commerce Operations</t>
         </is>
       </c>
       <c r="M10" s="4" t="inlineStr"/>
@@ -1458,7 +1454,7 @@
       </c>
       <c r="X10" s="5" t="inlineStr">
         <is>
-          <t>P2. Applied for Manager - Process Excellence May 2026. Established D2C, strong fit.</t>
+          <t>P3. Applied May 2026, no reply.</t>
         </is>
       </c>
     </row>
@@ -1466,17 +1462,17 @@
       <c r="A11" s="4" t="inlineStr"/>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Samplify</t>
+          <t>CitizenEarth</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>gosamplify.com</t>
+          <t>citizenearth.in</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>D2C / Sampling</t>
+          <t>D2C / Sustainability</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -1487,7 +1483,7 @@
       <c r="F11" s="4" t="inlineStr"/>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Hemlata</t>
+          <t>Hiring Team</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1497,7 +1493,7 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>hemlata@gosamplify.com</t>
+          <t>hr@citizenearth.in</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1512,7 +1508,7 @@
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>Team Lead - Operations</t>
+          <t>Operations Lead</t>
         </is>
       </c>
       <c r="M11" s="4" t="inlineStr"/>
@@ -1544,7 +1540,7 @@
       </c>
       <c r="X11" s="5" t="inlineStr">
         <is>
-          <t>P2. Applied May 2026, no reply.</t>
+          <t>P4. Generic HR alias. Applied May 2026, no reply.</t>
         </is>
       </c>
     </row>
@@ -1552,38 +1548,38 @@
       <c r="A12" s="4" t="inlineStr"/>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>goPortals</t>
+          <t>iCARRY</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>goportals.co</t>
+          <t>icarry.com</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>E-commerce</t>
+          <t>Logistics / E-commerce</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Early</t>
+          <t>Growth</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr"/>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Sahil Gupta</t>
+          <t>Talent Team</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Founder</t>
+          <t>Talent</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>sahilgupta@goportals.co</t>
+          <t>Talents@icarry.com</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -1598,7 +1594,7 @@
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t>E-commerce Operations</t>
+          <t>Operations Manager</t>
         </is>
       </c>
       <c r="M12" s="4" t="inlineStr"/>
@@ -1629,178 +1625,6 @@
         </is>
       </c>
       <c r="X12" s="5" t="inlineStr">
-        <is>
-          <t>P3. Applied May 2026, no reply.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr"/>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>CitizenEarth</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>citizenearth.in</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>D2C / Sustainability</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>Early</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr"/>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>Hiring Team</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>HR</t>
-        </is>
-      </c>
-      <c r="I13" s="4" t="inlineStr">
-        <is>
-          <t>hr@citizenearth.in</t>
-        </is>
-      </c>
-      <c r="J13" s="4" t="inlineStr">
-        <is>
-          <t>Gmail - outbound May 2026</t>
-        </is>
-      </c>
-      <c r="K13" s="4" t="inlineStr">
-        <is>
-          <t>Cold</t>
-        </is>
-      </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>Operations Lead</t>
-        </is>
-      </c>
-      <c r="M13" s="4" t="inlineStr"/>
-      <c r="N13" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O13" s="4" t="inlineStr"/>
-      <c r="P13" s="4" t="inlineStr"/>
-      <c r="Q13" s="4" t="inlineStr"/>
-      <c r="R13" s="4" t="inlineStr"/>
-      <c r="S13" s="4" t="inlineStr"/>
-      <c r="T13" s="4" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="U13" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="V13" s="4" t="inlineStr"/>
-      <c r="W13" s="4" t="inlineStr">
-        <is>
-          <t>Ready to Send</t>
-        </is>
-      </c>
-      <c r="X13" s="5" t="inlineStr">
-        <is>
-          <t>P4. Generic HR alias. Applied May 2026, no reply.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr"/>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>iCARRY</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>icarry.com</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>Logistics / E-commerce</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>Growth</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr"/>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>Talent Team</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>Talent</t>
-        </is>
-      </c>
-      <c r="I14" s="4" t="inlineStr">
-        <is>
-          <t>Talents@icarry.com</t>
-        </is>
-      </c>
-      <c r="J14" s="4" t="inlineStr">
-        <is>
-          <t>Gmail - outbound May 2026</t>
-        </is>
-      </c>
-      <c r="K14" s="4" t="inlineStr">
-        <is>
-          <t>Cold</t>
-        </is>
-      </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>Operations Manager</t>
-        </is>
-      </c>
-      <c r="M14" s="4" t="inlineStr"/>
-      <c r="N14" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O14" s="4" t="inlineStr"/>
-      <c r="P14" s="4" t="inlineStr"/>
-      <c r="Q14" s="4" t="inlineStr"/>
-      <c r="R14" s="4" t="inlineStr"/>
-      <c r="S14" s="4" t="inlineStr"/>
-      <c r="T14" s="4" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="U14" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="V14" s="4" t="inlineStr"/>
-      <c r="W14" s="4" t="inlineStr">
-        <is>
-          <t>Ready to Send</t>
-        </is>
-      </c>
-      <c r="X14" s="5" t="inlineStr">
         <is>
           <t>P4. Generic alias. Logistics OS for emerging markets - good ops fit.</t>
         </is>

</xml_diff>

<commit_message>
Add five D2C brand contacts from company careers pages
Every address read directly off the company's own site. Two carry a live
role match: Earthful (quick commerce manager) and The Wellness Shop
(head of operations, supply chain).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TsefmjrgrWVU5PNpRHnLLk
</commit_message>
<xml_diff>
--- a/outreach/Outreach_Tracker.xlsx
+++ b/outreach/Outreach_Tracker.xlsx
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X12"/>
+  <dimension ref="A1:X17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1627,6 +1627,452 @@
       <c r="X12" s="5" t="inlineStr">
         <is>
           <t>P4. Generic alias. Logistics OS for emerging markets - good ops fit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr"/>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>TruNativ</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>trunativ.co</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>D2C / Nutrition</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Growth</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Mumbai (Andheri W)</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Talent Team</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Recruitment</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>talent@trunativ.co</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>Careers page - trunativ.co/pages/careers</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>Operations Manager</t>
+        </is>
+      </c>
+      <c r="M13" s="4" t="inlineStr"/>
+      <c r="N13" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O13" s="4" t="inlineStr"/>
+      <c r="P13" s="4" t="inlineStr"/>
+      <c r="Q13" s="4" t="inlineStr"/>
+      <c r="R13" s="4" t="inlineStr"/>
+      <c r="S13" s="4" t="inlineStr"/>
+      <c r="T13" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="U13" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V13" s="4" t="inlineStr"/>
+      <c r="W13" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Send</t>
+        </is>
+      </c>
+      <c r="X13" s="5" t="inlineStr">
+        <is>
+          <t>P2. Careers page says explicitly "Send your profile to talent@trunativ.co". Purpose-built recruitment inbox, no role advertised - speculative application.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr"/>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Wellbeing Nutrition</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>wellbeingnutrition.com</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>D2C / Nutrition</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Growth</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Gurgaon</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>Talent Team</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>talent@wellbeingnutrition.com</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>Careers page - wellbeingnutrition.com/pages/careers</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>Operations Manager</t>
+        </is>
+      </c>
+      <c r="M14" s="4" t="inlineStr"/>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O14" s="4" t="inlineStr"/>
+      <c r="P14" s="4" t="inlineStr"/>
+      <c r="Q14" s="4" t="inlineStr"/>
+      <c r="R14" s="4" t="inlineStr"/>
+      <c r="S14" s="4" t="inlineStr"/>
+      <c r="T14" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="U14" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V14" s="4" t="inlineStr"/>
+      <c r="W14" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Send</t>
+        </is>
+      </c>
+      <c r="X14" s="5" t="inlineStr">
+        <is>
+          <t>P2. HR email on careers page. 300+ SKUs, owns full supply chain, 600+ retail doors alongside D2C - strong profile fit. No ops role advertised; open roles are marketing/design.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr"/>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Earthful</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>earthful.me</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>D2C / Nutrition</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Early</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Hyderabad / Mumbai</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Care Team</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>care@earthful.me</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>Careers page - earthful.me/pages/careers</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Quick Commerce Manager</t>
+        </is>
+      </c>
+      <c r="M15" s="4" t="inlineStr"/>
+      <c r="N15" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O15" s="4" t="inlineStr"/>
+      <c r="P15" s="4" t="inlineStr"/>
+      <c r="Q15" s="4" t="inlineStr"/>
+      <c r="R15" s="4" t="inlineStr"/>
+      <c r="S15" s="4" t="inlineStr"/>
+      <c r="T15" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="U15" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V15" s="4" t="inlineStr"/>
+      <c r="W15" s="4" t="inlineStr">
+        <is>
+          <t>Researching</t>
+        </is>
+      </c>
+      <c r="X15" s="5" t="inlineStr">
+        <is>
+          <t>P1 ROLE MATCH. Hiring "Quick Commerce Manager (Blinkit, Zepto, Swiggy Instamart)" - exact Sova Health experience. Apply via the on-site form, NOT this address (care@ is customer support). Use quick-commerce wording for this one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr"/>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>The Wellness Shop</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>thewellnessshop.in</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>D2C / Wellness</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Growth</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr"/>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Care Team</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>care@thewellnessshop.in</t>
+        </is>
+      </c>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>Contact page - thewellnessshop.in</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>Head - Operations, Supply Chain</t>
+        </is>
+      </c>
+      <c r="M16" s="4" t="inlineStr"/>
+      <c r="N16" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O16" s="4" t="inlineStr"/>
+      <c r="P16" s="4" t="inlineStr"/>
+      <c r="Q16" s="4" t="inlineStr"/>
+      <c r="R16" s="4" t="inlineStr"/>
+      <c r="S16" s="4" t="inlineStr"/>
+      <c r="T16" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="U16" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V16" s="4" t="inlineStr"/>
+      <c r="W16" s="4" t="inlineStr">
+        <is>
+          <t>Researching</t>
+        </is>
+      </c>
+      <c r="X16" s="5" t="inlineStr">
+        <is>
+          <t>P2 ROLE MATCH. iimjobs lists "Head - Operations, Supply Chain/Warehouse &amp; Logistics, D2C eCommerce" (login needed to view). Careers page has an Apply Now form and no HR email; care@ is customer support. Apply via form or iimjobs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr"/>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>BeastLife</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>beastlife.in</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>D2C / Sports Nutrition</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Growth</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Gurugram</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Care Team</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>care@beastlife.in</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>Contact page - beastlife.in/pages/contact</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Operations Manager</t>
+        </is>
+      </c>
+      <c r="M17" s="4" t="inlineStr"/>
+      <c r="N17" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O17" s="4" t="inlineStr"/>
+      <c r="P17" s="4" t="inlineStr"/>
+      <c r="Q17" s="4" t="inlineStr"/>
+      <c r="R17" s="4" t="inlineStr"/>
+      <c r="S17" s="4" t="inlineStr"/>
+      <c r="T17" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="U17" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V17" s="4" t="inlineStr"/>
+      <c r="W17" s="4" t="inlineStr">
+        <is>
+          <t>Researching</t>
+        </is>
+      </c>
+      <c r="X17" s="5" t="inlineStr">
+        <is>
+          <t>P4. No careers page and no HR email published; care@ is customer support. RAK Fitness Consumer Pvt Ltd, Udyog Vihar Phase 1. Low-yield - try LinkedIn for a named contact first.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Earthful, Wellness Shop and BeastLife applications
Three role-matched emails that keep the quick-commerce wording, since the
Blinkit/Zepto/Instamart experience is the point of the match. BeastLife
contact updated to the address Aditya supplied.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TsefmjrgrWVU5PNpRHnLLk
</commit_message>
<xml_diff>
--- a/outreach/Outreach_Tracker.xlsx
+++ b/outreach/Outreach_Tracker.xlsx
@@ -2015,22 +2015,22 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Care Team</t>
+          <t>Raj</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Hiring Contact</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>care@beastlife.in</t>
+          <t>raj@beastlife.in</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>Contact page - beastlife.in/pages/contact</t>
+          <t>Provided by Aditya</t>
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr">
@@ -2067,12 +2067,12 @@
       <c r="V17" s="4" t="inlineStr"/>
       <c r="W17" s="4" t="inlineStr">
         <is>
-          <t>Researching</t>
+          <t>Ready to Send</t>
         </is>
       </c>
       <c r="X17" s="5" t="inlineStr">
         <is>
-          <t>P4. No careers page and no HR email published; care@ is customer support. RAK Fitness Consumer Pvt Ltd, Udyog Vihar Phase 1. Low-yield - try LinkedIn for a named contact first.</t>
+          <t>P2. Named contact supplied by Aditya. No careers page on site; RAK Fitness Consumer Pvt Ltd, Udyog Vihar Phase 1, Gurugram.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mark the 24 Aug batch as sent
All 14 emails sent at 11:30 IST. TruNativ and Wellbeing Nutrition stay
Ready to Send - no email has been written for either yet.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TsefmjrgrWVU5PNpRHnLLk
</commit_message>
<xml_diff>
--- a/outreach/Outreach_Tracker.xlsx
+++ b/outreach/Outreach_Tracker.xlsx
@@ -669,7 +669,11 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
           <t>The Bijou Box</t>
@@ -725,17 +729,33 @@
           <t>E-commerce Operations</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Re-opening my application — E-commerce Operations, The Bijou Box</t>
+        </is>
+      </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr"/>
-      <c r="P2" s="2" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Q2" s="2" t="inlineStr"/>
       <c r="R2" s="2" t="inlineStr"/>
-      <c r="S2" s="2" t="inlineStr"/>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -749,7 +769,7 @@
       <c r="V2" s="2" t="inlineStr"/>
       <c r="W2" s="2" t="inlineStr">
         <is>
-          <t>Ready to Send</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="X2" s="3" t="inlineStr">
@@ -759,7 +779,11 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Gudz</t>
@@ -815,17 +839,33 @@
           <t>Operations Manager</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Following up, at operations manager level — Aditya Kumar</t>
+        </is>
+      </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O3" s="2" t="inlineStr"/>
-      <c r="P3" s="2" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Q3" s="2" t="inlineStr"/>
       <c r="R3" s="2" t="inlineStr"/>
-      <c r="S3" s="2" t="inlineStr"/>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -839,7 +879,7 @@
       <c r="V3" s="2" t="inlineStr"/>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>Ready to Send</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="X3" s="3" t="inlineStr">
@@ -849,7 +889,11 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr"/>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Meesho</t>
@@ -905,17 +949,33 @@
           <t>Area Manager / Ops</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Area Manager / Operations — following up on my application</t>
+        </is>
+      </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O4" s="2" t="inlineStr"/>
-      <c r="P4" s="2" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Q4" s="2" t="inlineStr"/>
       <c r="R4" s="2" t="inlineStr"/>
-      <c r="S4" s="2" t="inlineStr"/>
+      <c r="S4" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -929,7 +989,7 @@
       <c r="V4" s="2" t="inlineStr"/>
       <c r="W4" s="2" t="inlineStr">
         <is>
-          <t>Ready to Send</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="X4" s="3" t="inlineStr">
@@ -939,7 +999,11 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Elda</t>
@@ -991,17 +1055,33 @@
           <t>Business Operations</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>Business Operations at Elda — following up beyond the intern role</t>
+        </is>
+      </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O5" s="2" t="inlineStr"/>
-      <c r="P5" s="2" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Q5" s="2" t="inlineStr"/>
       <c r="R5" s="2" t="inlineStr"/>
-      <c r="S5" s="2" t="inlineStr"/>
+      <c r="S5" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -1015,7 +1095,7 @@
       <c r="V5" s="2" t="inlineStr"/>
       <c r="W5" s="2" t="inlineStr">
         <is>
-          <t>Ready to Send</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="X5" s="3" t="inlineStr">
@@ -1025,7 +1105,11 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr"/>
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Cameron SF</t>
@@ -1077,17 +1161,33 @@
           <t>Operations Manager</t>
         </is>
       </c>
-      <c r="M6" s="4" t="inlineStr"/>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
+          <t>Operations Manager — following up on my application</t>
+        </is>
+      </c>
       <c r="N6" s="4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O6" s="4" t="inlineStr"/>
-      <c r="P6" s="4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O6" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="P6" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Q6" s="4" t="inlineStr"/>
       <c r="R6" s="4" t="inlineStr"/>
-      <c r="S6" s="4" t="inlineStr"/>
+      <c r="S6" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="T6" s="4" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -1101,7 +1201,7 @@
       <c r="V6" s="4" t="inlineStr"/>
       <c r="W6" s="4" t="inlineStr">
         <is>
-          <t>Ready to Send</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="X6" s="5" t="inlineStr">
@@ -1111,7 +1211,11 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr"/>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Zoomuv</t>
@@ -1163,17 +1267,33 @@
           <t>Operations Executive</t>
         </is>
       </c>
-      <c r="M7" s="4" t="inlineStr"/>
+      <c r="M7" s="4" t="inlineStr">
+        <is>
+          <t>Operations at Zoomuv — dispatch SLA, inventory control, process automation</t>
+        </is>
+      </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O7" s="4" t="inlineStr"/>
-      <c r="P7" s="4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O7" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="P7" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Q7" s="4" t="inlineStr"/>
       <c r="R7" s="4" t="inlineStr"/>
-      <c r="S7" s="4" t="inlineStr"/>
+      <c r="S7" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="T7" s="4" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -1187,7 +1307,7 @@
       <c r="V7" s="4" t="inlineStr"/>
       <c r="W7" s="4" t="inlineStr">
         <is>
-          <t>Ready to Send</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="X7" s="5" t="inlineStr">
@@ -1197,7 +1317,11 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr"/>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Ugaoo</t>
@@ -1253,17 +1377,33 @@
           <t>Operations Manager</t>
         </is>
       </c>
-      <c r="M8" s="4" t="inlineStr"/>
+      <c r="M8" s="4" t="inlineStr">
+        <is>
+          <t>Operations Manager — 98%+ dispatch SLA on perishable, high-RTO categories</t>
+        </is>
+      </c>
       <c r="N8" s="4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O8" s="4" t="inlineStr"/>
-      <c r="P8" s="4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O8" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="P8" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Q8" s="4" t="inlineStr"/>
       <c r="R8" s="4" t="inlineStr"/>
-      <c r="S8" s="4" t="inlineStr"/>
+      <c r="S8" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="T8" s="4" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -1277,7 +1417,7 @@
       <c r="V8" s="4" t="inlineStr"/>
       <c r="W8" s="4" t="inlineStr">
         <is>
-          <t>Ready to Send</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="X8" s="5" t="inlineStr">
@@ -1287,7 +1427,11 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr"/>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Samplify</t>
@@ -1339,17 +1483,33 @@
           <t>Team Lead - Operations</t>
         </is>
       </c>
-      <c r="M9" s="4" t="inlineStr"/>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
+          <t>Team Lead, Operations — scaled e-commerce from INR 50L to 4.3 Cr in 8 months</t>
+        </is>
+      </c>
       <c r="N9" s="4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O9" s="4" t="inlineStr"/>
-      <c r="P9" s="4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O9" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="P9" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Q9" s="4" t="inlineStr"/>
       <c r="R9" s="4" t="inlineStr"/>
-      <c r="S9" s="4" t="inlineStr"/>
+      <c r="S9" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="T9" s="4" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -1363,7 +1523,7 @@
       <c r="V9" s="4" t="inlineStr"/>
       <c r="W9" s="4" t="inlineStr">
         <is>
-          <t>Ready to Send</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="X9" s="5" t="inlineStr">
@@ -1373,7 +1533,11 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr"/>
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
           <t>goPortals</t>
@@ -1425,17 +1589,33 @@
           <t>E-commerce Operations</t>
         </is>
       </c>
-      <c r="M10" s="4" t="inlineStr"/>
+      <c r="M10" s="4" t="inlineStr">
+        <is>
+          <t>E-commerce Operations — marketplace dispatch, inventory reconciliation</t>
+        </is>
+      </c>
       <c r="N10" s="4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O10" s="4" t="inlineStr"/>
-      <c r="P10" s="4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O10" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="P10" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Q10" s="4" t="inlineStr"/>
       <c r="R10" s="4" t="inlineStr"/>
-      <c r="S10" s="4" t="inlineStr"/>
+      <c r="S10" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="T10" s="4" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -1449,7 +1629,7 @@
       <c r="V10" s="4" t="inlineStr"/>
       <c r="W10" s="4" t="inlineStr">
         <is>
-          <t>Ready to Send</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="X10" s="5" t="inlineStr">
@@ -1459,7 +1639,11 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr"/>
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
           <t>CitizenEarth</t>
@@ -1511,17 +1695,33 @@
           <t>Operations Lead</t>
         </is>
       </c>
-      <c r="M11" s="4" t="inlineStr"/>
+      <c r="M11" s="4" t="inlineStr">
+        <is>
+          <t>Operations Lead — D2C dispatch, inventory control, 98%+ SLA</t>
+        </is>
+      </c>
       <c r="N11" s="4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O11" s="4" t="inlineStr"/>
-      <c r="P11" s="4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O11" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="P11" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Q11" s="4" t="inlineStr"/>
       <c r="R11" s="4" t="inlineStr"/>
-      <c r="S11" s="4" t="inlineStr"/>
+      <c r="S11" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="T11" s="4" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -1535,7 +1735,7 @@
       <c r="V11" s="4" t="inlineStr"/>
       <c r="W11" s="4" t="inlineStr">
         <is>
-          <t>Ready to Send</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="X11" s="5" t="inlineStr">
@@ -1545,7 +1745,11 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr"/>
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
           <t>iCARRY</t>
@@ -1597,17 +1801,33 @@
           <t>Operations Manager</t>
         </is>
       </c>
-      <c r="M12" s="4" t="inlineStr"/>
+      <c r="M12" s="4" t="inlineStr">
+        <is>
+          <t>Operations Manager — inventory and dispatch, 98%+ SLA across marketplaces</t>
+        </is>
+      </c>
       <c r="N12" s="4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O12" s="4" t="inlineStr"/>
-      <c r="P12" s="4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O12" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="P12" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Q12" s="4" t="inlineStr"/>
       <c r="R12" s="4" t="inlineStr"/>
-      <c r="S12" s="4" t="inlineStr"/>
+      <c r="S12" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="T12" s="4" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -1621,7 +1841,7 @@
       <c r="V12" s="4" t="inlineStr"/>
       <c r="W12" s="4" t="inlineStr">
         <is>
-          <t>Ready to Send</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="X12" s="5" t="inlineStr">
@@ -1811,7 +2031,11 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr"/>
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Earthful</t>
@@ -1867,17 +2091,33 @@
           <t>Quick Commerce Manager</t>
         </is>
       </c>
-      <c r="M15" s="4" t="inlineStr"/>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>Quick Commerce Manager — scaled Blinkit, Zepto and Instamart from INR 50L to 4.3 Cr in 8 months</t>
+        </is>
+      </c>
       <c r="N15" s="4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O15" s="4" t="inlineStr"/>
-      <c r="P15" s="4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O15" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="P15" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Q15" s="4" t="inlineStr"/>
       <c r="R15" s="4" t="inlineStr"/>
-      <c r="S15" s="4" t="inlineStr"/>
+      <c r="S15" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="T15" s="4" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -1891,7 +2131,7 @@
       <c r="V15" s="4" t="inlineStr"/>
       <c r="W15" s="4" t="inlineStr">
         <is>
-          <t>Researching</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="X15" s="5" t="inlineStr">
@@ -1901,7 +2141,11 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr"/>
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
           <t>The Wellness Shop</t>
@@ -1953,17 +2197,33 @@
           <t>Head - Operations, Supply Chain</t>
         </is>
       </c>
-      <c r="M16" s="4" t="inlineStr"/>
+      <c r="M16" s="4" t="inlineStr">
+        <is>
+          <t>Head of Operations, Supply Chain and Logistics — 98%+ dispatch SLA, zero stockouts</t>
+        </is>
+      </c>
       <c r="N16" s="4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O16" s="4" t="inlineStr"/>
-      <c r="P16" s="4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O16" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="P16" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Q16" s="4" t="inlineStr"/>
       <c r="R16" s="4" t="inlineStr"/>
-      <c r="S16" s="4" t="inlineStr"/>
+      <c r="S16" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="T16" s="4" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -1977,7 +2237,7 @@
       <c r="V16" s="4" t="inlineStr"/>
       <c r="W16" s="4" t="inlineStr">
         <is>
-          <t>Researching</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="X16" s="5" t="inlineStr">
@@ -1987,7 +2247,11 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr"/>
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
           <t>BeastLife</t>
@@ -2043,17 +2307,33 @@
           <t>Operations Manager</t>
         </is>
       </c>
-      <c r="M17" s="4" t="inlineStr"/>
+      <c r="M17" s="4" t="inlineStr">
+        <is>
+          <t>Operations Manager — inventory, dispatch and quick commerce for a scaling D2C brand</t>
+        </is>
+      </c>
       <c r="N17" s="4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O17" s="4" t="inlineStr"/>
-      <c r="P17" s="4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O17" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="P17" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Q17" s="4" t="inlineStr"/>
       <c r="R17" s="4" t="inlineStr"/>
-      <c r="S17" s="4" t="inlineStr"/>
+      <c r="S17" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="T17" s="4" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -2067,7 +2347,7 @@
       <c r="V17" s="4" t="inlineStr"/>
       <c r="W17" s="4" t="inlineStr">
         <is>
-          <t>Ready to Send</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="X17" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Add recruitment agency outreach and Pebble application
Four staffing firms with logistics and SCM desks, plus Pebble, which is
advertising a D2C ops role on Shopify and Unicommerce. Agency emails carry a
placeholder for notice period and CTC, which are not in the CV sources.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TsefmjrgrWVU5PNpRHnLLk
</commit_message>
<xml_diff>
--- a/outreach/Outreach_Tracker.xlsx
+++ b/outreach/Outreach_Tracker.xlsx
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X17"/>
+  <dimension ref="A1:X22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2353,6 +2353,452 @@
       <c r="X17" s="5" t="inlineStr">
         <is>
           <t>P2. Named contact supplied by Aditya. No careers page on site; RAK Fitness Consumer Pvt Ltd, Udyog Vihar Phase 1, Gurugram.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr"/>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Prompt Personnel</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>promptpersonnel.com</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Recruitment Agency</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Established</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Mumbai (Malad W)</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>HR Team</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Recruitment</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>hr@promptpersonnel.com</t>
+        </is>
+      </c>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>Site - promptpersonnel.com/logistics-recruitment-agency</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>Operations / Inventory Manager</t>
+        </is>
+      </c>
+      <c r="M18" s="4" t="inlineStr"/>
+      <c r="N18" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O18" s="4" t="inlineStr"/>
+      <c r="P18" s="4" t="inlineStr"/>
+      <c r="Q18" s="4" t="inlineStr"/>
+      <c r="R18" s="4" t="inlineStr"/>
+      <c r="S18" s="4" t="inlineStr"/>
+      <c r="T18" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="U18" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V18" s="4" t="inlineStr"/>
+      <c r="W18" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Send</t>
+        </is>
+      </c>
+      <c r="X18" s="5" t="inlineStr">
+        <is>
+          <t>P2 AGENCY. Site labels this address "for job opportunities" - the only agency found with a dedicated candidate inbox. 25+ yrs, places Operations roles. Offices Mumbai, Delhi, Bengaluru, Chennai, Hyderabad, Kolkata.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr"/>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>WSNE Consulting</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>wsneconsulting.com</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Recruitment Agency</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Growth</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>New Delhi (Dwarka Mor)</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Recruitment</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>info@wsneconsulting.com</t>
+        </is>
+      </c>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>Site - wsneconsulting.com/sectors/logistics</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Operations / Inventory Manager</t>
+        </is>
+      </c>
+      <c r="M19" s="4" t="inlineStr"/>
+      <c r="N19" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O19" s="4" t="inlineStr"/>
+      <c r="P19" s="4" t="inlineStr"/>
+      <c r="Q19" s="4" t="inlineStr"/>
+      <c r="R19" s="4" t="inlineStr"/>
+      <c r="S19" s="4" t="inlineStr"/>
+      <c r="T19" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="U19" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V19" s="4" t="inlineStr"/>
+      <c r="W19" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Send</t>
+        </is>
+      </c>
+      <c r="X19" s="5" t="inlineStr">
+        <is>
+          <t>P3 AGENCY. Logistics and SCM specialists, claims 450+ logistics placements and 70+ SCM clients across e-commerce fulfilment, cold chain and 3PL. Delhi NCR based - good geography.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr"/>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Perito</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>perito.co.in</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Recruitment Agency</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Established</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Noida (Sector 63)</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>Recruitment</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>info@perito.co.in</t>
+        </is>
+      </c>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>Site - perito.co.in/sectors-catered/logistics</t>
+        </is>
+      </c>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>Operations / Dispatch Manager</t>
+        </is>
+      </c>
+      <c r="M20" s="4" t="inlineStr"/>
+      <c r="N20" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O20" s="4" t="inlineStr"/>
+      <c r="P20" s="4" t="inlineStr"/>
+      <c r="Q20" s="4" t="inlineStr"/>
+      <c r="R20" s="4" t="inlineStr"/>
+      <c r="S20" s="4" t="inlineStr"/>
+      <c r="T20" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="U20" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V20" s="4" t="inlineStr"/>
+      <c r="W20" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Send</t>
+        </is>
+      </c>
+      <c r="X20" s="5" t="inlineStr">
+        <is>
+          <t>P3 AGENCY. Logistics and transportation placement specialists. Head office Noida, offices in Delhi, Ghaziabad, Agra, Meerut, Kolkata.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr"/>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Futurz HR</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>futurzhr.com</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Recruitment Agency</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Established</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr"/>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Recruitment</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>info@futurzhr.com</t>
+        </is>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>Site - futurzhr.com/services/logistics-recruitment-agency</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Operations / Warehouse Manager</t>
+        </is>
+      </c>
+      <c r="M21" s="4" t="inlineStr"/>
+      <c r="N21" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O21" s="4" t="inlineStr"/>
+      <c r="P21" s="4" t="inlineStr"/>
+      <c r="Q21" s="4" t="inlineStr"/>
+      <c r="R21" s="4" t="inlineStr"/>
+      <c r="S21" s="4" t="inlineStr"/>
+      <c r="T21" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="U21" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V21" s="4" t="inlineStr"/>
+      <c r="W21" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Send</t>
+        </is>
+      </c>
+      <c r="X21" s="5" t="inlineStr">
+        <is>
+          <t>P3 AGENCY. Logistics staffing across supply chain, warehouse, transport and procurement. Places white-collar SCM roles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr"/>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Pebble</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>pebblecart.com</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>D2C / Consumer Electronics</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Growth</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Noida</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>Support Team</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>support@pebblecart.com</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>Contact page - pebblecart.com/pages/contact</t>
+        </is>
+      </c>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>D2C Operations Manager</t>
+        </is>
+      </c>
+      <c r="M22" s="4" t="inlineStr"/>
+      <c r="N22" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O22" s="4" t="inlineStr"/>
+      <c r="P22" s="4" t="inlineStr"/>
+      <c r="Q22" s="4" t="inlineStr"/>
+      <c r="R22" s="4" t="inlineStr"/>
+      <c r="S22" s="4" t="inlineStr"/>
+      <c r="T22" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="U22" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V22" s="4" t="inlineStr"/>
+      <c r="W22" s="4" t="inlineStr">
+        <is>
+          <t>Researching</t>
+        </is>
+      </c>
+      <c r="X22" s="5" t="inlineStr">
+        <is>
+          <t>P3 ROLE MATCH. Advertising a D2C Operations Manager running backend e-commerce ops on Shopify AND Unicommerce - both tools used at Sova. Posted Jul 2026. No careers page or HR email found; support@ is customer service. SRK Powertech Pvt Ltd, Advant Navis Park, Noida.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add UAE outreach and finalise agency emails
TASC Outsourcing and iStore for the UAE move; both state the visa
sponsorship requirement up front. CTC placeholder dropped from the agency
emails since those figures are not in the CV sources.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TsefmjrgrWVU5PNpRHnLLk
</commit_message>
<xml_diff>
--- a/outreach/Outreach_Tracker.xlsx
+++ b/outreach/Outreach_Tracker.xlsx
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X22"/>
+  <dimension ref="A1:X24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2799,6 +2799,186 @@
       <c r="X22" s="5" t="inlineStr">
         <is>
           <t>P3 ROLE MATCH. Advertising a D2C Operations Manager running backend e-commerce ops on Shopify AND Unicommerce - both tools used at Sova. Posted Jul 2026. No careers page or HR email found; support@ is customer service. SRK Powertech Pvt Ltd, Advant Navis Park, Noida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr"/>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>TASC Outsourcing</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>tascoutsourcing.com</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Recruitment Agency</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Established</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Dubai + Abu Dhabi</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Recruitment Team</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>CV Submissions</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>dxbjobs@tascoutsourcing.com</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>Site - tascoutsourcing.com/en/specialisations/logistics-supply-chain</t>
+        </is>
+      </c>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Operations / Inventory Manager (UAE)</t>
+        </is>
+      </c>
+      <c r="M23" s="4" t="inlineStr"/>
+      <c r="N23" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O23" s="4" t="inlineStr"/>
+      <c r="P23" s="4" t="inlineStr"/>
+      <c r="Q23" s="4" t="inlineStr"/>
+      <c r="R23" s="4" t="inlineStr"/>
+      <c r="S23" s="4" t="inlineStr"/>
+      <c r="T23" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="U23" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V23" s="4" t="inlineStr"/>
+      <c r="W23" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Send</t>
+        </is>
+      </c>
+      <c r="X23" s="5" t="inlineStr">
+        <is>
+          <t>P2 AGENCY UAE. Only UAE firm found publishing a real CV-submission address. Logistics and SCM desk, 15+ yrs MENA. Dubai HQ Nassima Tower plus Abu Dhabi office. Also register at tascoutsourcing.com/en/candidates/register-cv.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr"/>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>iStore</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>istoreae.com</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>3PL / E-commerce Fulfilment</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Growth</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Ajman, UAE</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>info@istoreae.com</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>Site - istoreae.com/warehouse-fulfillment-uae</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Operations / Inventory Manager (UAE)</t>
+        </is>
+      </c>
+      <c r="M24" s="4" t="inlineStr"/>
+      <c r="N24" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O24" s="4" t="inlineStr"/>
+      <c r="P24" s="4" t="inlineStr"/>
+      <c r="Q24" s="4" t="inlineStr"/>
+      <c r="R24" s="4" t="inlineStr"/>
+      <c r="S24" s="4" t="inlineStr"/>
+      <c r="T24" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="U24" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V24" s="4" t="inlineStr"/>
+      <c r="W24" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Send</t>
+        </is>
+      </c>
+      <c r="X24" s="5" t="inlineStr">
+        <is>
+          <t>P4 UAE. E-commerce fulfilment and 3PL warehousing. Only a general info@ inbox published, no careers page. Ajman rather than Dubai or Abu Dhabi.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mark the 25 Aug batch as sent
Seven sent at 10:30 IST: four Indian agencies, Pebble, and the two UAE
contacts. Tracked as a separate block from the 24 Aug batch.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TsefmjrgrWVU5PNpRHnLLk
</commit_message>
<xml_diff>
--- a/outreach/Outreach_Tracker.xlsx
+++ b/outreach/Outreach_Tracker.xlsx
@@ -2357,7 +2357,11 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr"/>
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Prompt Personnel</t>
@@ -2413,17 +2417,33 @@
           <t>Operations / Inventory Manager</t>
         </is>
       </c>
-      <c r="M18" s="4" t="inlineStr"/>
+      <c r="M18" s="4" t="inlineStr">
+        <is>
+          <t>Operations and Inventory Manager, 4+ years — registering for D2C and supply chain mandates</t>
+        </is>
+      </c>
       <c r="N18" s="4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O18" s="4" t="inlineStr"/>
-      <c r="P18" s="4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O18" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="P18" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr"/>
-      <c r="S18" s="4" t="inlineStr"/>
+      <c r="S18" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
       <c r="T18" s="4" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -2437,7 +2457,7 @@
       <c r="V18" s="4" t="inlineStr"/>
       <c r="W18" s="4" t="inlineStr">
         <is>
-          <t>Ready to Send</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="X18" s="5" t="inlineStr">
@@ -2447,7 +2467,11 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr"/>
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
           <t>WSNE Consulting</t>
@@ -2503,17 +2527,33 @@
           <t>Operations / Inventory Manager</t>
         </is>
       </c>
-      <c r="M19" s="4" t="inlineStr"/>
+      <c r="M19" s="4" t="inlineStr">
+        <is>
+          <t>Operations and Inventory Manager, 4+ years — registering for supply chain mandates</t>
+        </is>
+      </c>
       <c r="N19" s="4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O19" s="4" t="inlineStr"/>
-      <c r="P19" s="4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O19" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="P19" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Q19" s="4" t="inlineStr"/>
       <c r="R19" s="4" t="inlineStr"/>
-      <c r="S19" s="4" t="inlineStr"/>
+      <c r="S19" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
       <c r="T19" s="4" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -2527,7 +2567,7 @@
       <c r="V19" s="4" t="inlineStr"/>
       <c r="W19" s="4" t="inlineStr">
         <is>
-          <t>Ready to Send</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="X19" s="5" t="inlineStr">
@@ -2537,7 +2577,11 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr"/>
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
           <t>Perito</t>
@@ -2593,17 +2637,33 @@
           <t>Operations / Dispatch Manager</t>
         </is>
       </c>
-      <c r="M20" s="4" t="inlineStr"/>
+      <c r="M20" s="4" t="inlineStr">
+        <is>
+          <t>Operations and Inventory Manager, 4+ years — registering for supply chain mandates</t>
+        </is>
+      </c>
       <c r="N20" s="4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O20" s="4" t="inlineStr"/>
-      <c r="P20" s="4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O20" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="P20" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Q20" s="4" t="inlineStr"/>
       <c r="R20" s="4" t="inlineStr"/>
-      <c r="S20" s="4" t="inlineStr"/>
+      <c r="S20" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
       <c r="T20" s="4" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -2617,7 +2677,7 @@
       <c r="V20" s="4" t="inlineStr"/>
       <c r="W20" s="4" t="inlineStr">
         <is>
-          <t>Ready to Send</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="X20" s="5" t="inlineStr">
@@ -2627,7 +2687,11 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr"/>
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
           <t>Futurz HR</t>
@@ -2679,17 +2743,33 @@
           <t>Operations / Warehouse Manager</t>
         </is>
       </c>
-      <c r="M21" s="4" t="inlineStr"/>
+      <c r="M21" s="4" t="inlineStr">
+        <is>
+          <t>Operations and Inventory Manager, 4+ years — registering for supply chain mandates</t>
+        </is>
+      </c>
       <c r="N21" s="4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O21" s="4" t="inlineStr"/>
-      <c r="P21" s="4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O21" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="P21" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Q21" s="4" t="inlineStr"/>
       <c r="R21" s="4" t="inlineStr"/>
-      <c r="S21" s="4" t="inlineStr"/>
+      <c r="S21" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
       <c r="T21" s="4" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -2703,7 +2783,7 @@
       <c r="V21" s="4" t="inlineStr"/>
       <c r="W21" s="4" t="inlineStr">
         <is>
-          <t>Ready to Send</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="X21" s="5" t="inlineStr">
@@ -2713,7 +2793,11 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr"/>
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
           <t>Pebble</t>
@@ -2769,17 +2853,33 @@
           <t>D2C Operations Manager</t>
         </is>
       </c>
-      <c r="M22" s="4" t="inlineStr"/>
+      <c r="M22" s="4" t="inlineStr">
+        <is>
+          <t>D2C Operations Manager application — Shopify and Unicommerce, 98%+ dispatch SLA</t>
+        </is>
+      </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O22" s="4" t="inlineStr"/>
-      <c r="P22" s="4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O22" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="P22" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Q22" s="4" t="inlineStr"/>
       <c r="R22" s="4" t="inlineStr"/>
-      <c r="S22" s="4" t="inlineStr"/>
+      <c r="S22" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
       <c r="T22" s="4" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -2793,7 +2893,7 @@
       <c r="V22" s="4" t="inlineStr"/>
       <c r="W22" s="4" t="inlineStr">
         <is>
-          <t>Researching</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="X22" s="5" t="inlineStr">
@@ -2803,7 +2903,11 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr"/>
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
           <t>TASC Outsourcing</t>
@@ -2859,17 +2963,33 @@
           <t>Operations / Inventory Manager (UAE)</t>
         </is>
       </c>
-      <c r="M23" s="4" t="inlineStr"/>
+      <c r="M23" s="4" t="inlineStr">
+        <is>
+          <t>CV submission — Operations, Inventory and Dispatch Manager, 4+ years, relocating to UAE</t>
+        </is>
+      </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O23" s="4" t="inlineStr"/>
-      <c r="P23" s="4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O23" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="P23" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Q23" s="4" t="inlineStr"/>
       <c r="R23" s="4" t="inlineStr"/>
-      <c r="S23" s="4" t="inlineStr"/>
+      <c r="S23" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
       <c r="T23" s="4" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -2883,7 +3003,7 @@
       <c r="V23" s="4" t="inlineStr"/>
       <c r="W23" s="4" t="inlineStr">
         <is>
-          <t>Ready to Send</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="X23" s="5" t="inlineStr">
@@ -2893,7 +3013,11 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr"/>
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
           <t>iStore</t>
@@ -2949,17 +3073,33 @@
           <t>Operations / Inventory Manager (UAE)</t>
         </is>
       </c>
-      <c r="M24" s="4" t="inlineStr"/>
+      <c r="M24" s="4" t="inlineStr">
+        <is>
+          <t>Operations and Inventory Manager — e-commerce fulfilment, relocating to UAE</t>
+        </is>
+      </c>
       <c r="N24" s="4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O24" s="4" t="inlineStr"/>
-      <c r="P24" s="4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O24" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="P24" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="Q24" s="4" t="inlineStr"/>
       <c r="R24" s="4" t="inlineStr"/>
-      <c r="S24" s="4" t="inlineStr"/>
+      <c r="S24" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
       <c r="T24" s="4" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -2973,7 +3113,7 @@
       <c r="V24" s="4" t="inlineStr"/>
       <c r="W24" s="4" t="inlineStr">
         <is>
-          <t>Ready to Send</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="X24" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Record the goPortals and Earthful replies
goPortals asked for salary and Aditya answered directly. Earthful redirected
the application to hr@earthful.me, which has now been sent.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TsefmjrgrWVU5PNpRHnLLk
</commit_message>
<xml_diff>
--- a/outreach/Outreach_Tracker.xlsx
+++ b/outreach/Outreach_Tracker.xlsx
@@ -1609,8 +1609,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q10" s="4" t="inlineStr"/>
-      <c r="R10" s="4" t="inlineStr"/>
+      <c r="Q10" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R10" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
       <c r="S10" s="4" t="inlineStr">
         <is>
           <t>2026-09-01</t>
@@ -1629,12 +1637,12 @@
       <c r="V10" s="4" t="inlineStr"/>
       <c r="W10" s="4" t="inlineStr">
         <is>
-          <t>Sent</t>
+          <t>Replied</t>
         </is>
       </c>
       <c r="X10" s="5" t="inlineStr">
         <is>
-          <t>P3. Applied May 2026, no reply.</t>
+          <t>Sahil Gupta replied same day asking current and expected salary. Aditya answered directly: current 4.8 LPA / 40k in hand, expected 5.25 LPA fixed. NOTE: agency emails quote 9.0 LPA expected - figures differ. | P3. Applied May 2026, no reply.</t>
         </is>
       </c>
     </row>
@@ -2111,8 +2119,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="Q15" s="4" t="inlineStr"/>
-      <c r="R15" s="4" t="inlineStr"/>
+      <c r="Q15" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R15" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
           <t>2026-09-01</t>
@@ -2131,12 +2147,12 @@
       <c r="V15" s="4" t="inlineStr"/>
       <c r="W15" s="4" t="inlineStr">
         <is>
-          <t>Sent</t>
+          <t>Replied</t>
         </is>
       </c>
       <c r="X15" s="5" t="inlineStr">
         <is>
-          <t>P1 ROLE MATCH. Hiring "Quick Commerce Manager (Blinkit, Zepto, Swiggy Instamart)" - exact Sova Health experience. Apply via the on-site form, NOT this address (care@ is customer support). Use quick-commerce wording for this one.</t>
+          <t>Auto-reply from care@ redirected the application to hr@earthful.me. Re-sent there 25 Aug with full profile, notice period and current CTC. Careers page: earthful.me/pages/careers. | P1 ROLE MATCH. Hiring "Quick Commerce Manager (Blinkit, Zepto, Swiggy Instamart)" - exact Sova Health experience. Apply via the on-site form, NOT this address (care@ is customer support). Use quick-commerce wording for this one.</t>
         </is>
       </c>
     </row>

</xml_diff>